<commit_message>
Sprint 21: números honestos e repositório coerente
- Relatório mensal, lâminas 2 e 3 e doc de negócio abrem por indicadores
  relativos (serviço 60%→95%, ruptura −87%, capital +284%); R$ absolutos
  rotulados como ilustrativos (preço uniforme de R$ 10, margem arbitrada)
- Aviso de valores ilustrativos nas abas de detalhe do relatório mensal
- CLAUDE.md: emenda da Sprint 21 sobre as guardas (4 implementadas na
  Etapa 3.16) e sobre os R$ ilustrativos
- Notebooks renomeados por função (gerar_apresentacao, comparacao_*)
- Hooks do graphify movidos para .claude/settings.local.json (ignorado)
- docs/entregaveis regenerados a partir de results/
</commit_message>
<xml_diff>
--- a/docs/entregaveis/relatorio_mensal.xlsx
+++ b/docs/entregaveis/relatorio_mensal.xlsx
@@ -16,14 +16,14 @@
     <sheet name="Limitações" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Itens sangrando margem'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Itens sangrando margem'!$A$2:$J$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="148">
   <si>
     <t>RELATÓRIO MENSAL EM R$ -- MOTOR DE DECISÃO DE COMPRA</t>
   </si>
@@ -31,34 +31,46 @@
     <t>Período simulado avaliado: 2016-11-12 a 2017-08-15 (277 dias -- equivalente a 9.23 meses de 30 dias). Braço 2 (estatístico + nível-alvo), alpha=0.66 (iso-serviço). Célula lead_time=7/review_period=14 -- ver aba Premissas.</t>
   </si>
   <si>
+    <t>Indicadores relativos primeiro. Valores em R$: ilustrativo -- preço uniforme de R$ 10, margem arbitrada.</t>
+  </si>
+  <si>
     <t>ANDAR 1 -- CORREÇÃO DE CADASTRO (recalibrar, sem modelo)</t>
   </si>
   <si>
-    <t>Ruptura evitada (margem recuperada) -- mensal, magnitude calibrado_lt3_rp7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  faixa de sensibilidade de margem (±30%, mensal) -- ver aba Andar 1</t>
+    <t>Nível de serviço: de (calibrado_lt3_rp7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  para (baseline recalibrado)</t>
+  </si>
+  <si>
+    <t>Ruptura (R$) eliminada -- % da ruptura do baseline desatualizado</t>
+  </si>
+  <si>
+    <t>Custo: variação de capital médio empregado (recalibrar exige mais estoque, não libera; ver aba Andar 1)</t>
+  </si>
+  <si>
+    <t>Em R$ por mês -- ilustrativo -- preço uniforme de R$ 10, margem arbitrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ruptura evitada (margem recuperada), magnitude calibrado_lt3_rp7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  faixa de sensibilidade de margem (±30%) -- ver aba Andar 1</t>
   </si>
   <si>
     <t>132,973.38 a 246,950.57</t>
   </si>
   <si>
-    <t>Nível de serviço: de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  para (baseline recalibrado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  custo: aumento de capital empregado -- mensal (recalibrar exige mais estoque, não libera; ver aba Andar 1)</t>
+    <t xml:space="preserve">  aumento de capital empregado</t>
   </si>
   <si>
     <t>ANDAR 2 -- REFINAMENTO DO MODELO (sobre baseline já certo)</t>
   </si>
   <si>
-    <t>Capital liberado -- mensal (equivalente, ver nota)</t>
-  </si>
-  <si>
-    <t>Capital liberado -- % vs. baseline recalibrado (672,427.37)</t>
+    <t>Capital médio empregado -- variação vs. baseline recalibrado (negativo = libera)</t>
+  </si>
+  <si>
+    <t>Margem por real investido -- variação vs. baseline recalibrado</t>
   </si>
   <si>
     <t>decision_metric: baseline recalibrado</t>
@@ -67,7 +79,10 @@
     <t xml:space="preserve">  motor</t>
   </si>
   <si>
-    <t>Margem recuperada adicional pelo modelo -- mensal (pequena de propósito: mesmo nível de serviço do baseline recalibrado, por construção iso-serviço)</t>
+    <t xml:space="preserve">  capital liberado (equivalente, ver nota)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  margem recuperada adicional pelo modelo (pequena de propósito: mesmo nível de serviço do baseline recalibrado, por construção iso-serviço)</t>
   </si>
   <si>
     <t>Perda evitada (validade/expiração) -- os 2 andares</t>
@@ -83,6 +98,9 @@
   </si>
   <si>
     <t>O andar 1 abre a conta (não precisa de modelo); o andar 2 e a operação semanal da lista de compra são o que a mantêm -- ver Sprint 18.</t>
+  </si>
+  <si>
+    <t>Valores em R$: ilustrativo -- preço uniforme de R$ 10, margem arbitrada.</t>
   </si>
   <si>
     <t>indicador</t>
@@ -456,8 +474,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="3">
@@ -529,13 +547,13 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -830,7 +848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" customWidth="1"/>
@@ -847,117 +865,156 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
+    <row r="3" spans="1:2" ht="30" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <v>189961.9763693946</v>
-      </c>
+      <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
+      <c r="B6" s="4">
+        <v>0.59985842</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4">
-        <v>0.59985842</v>
+        <v>0.9485436</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="4">
-        <v>0.9485436</v>
+        <v>0.8687172826292039</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4">
+        <v>2.839951434445293</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3">
-        <v>53860.70717579459</v>
-      </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="5">
+        <v>189961.9763693946</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3">
-        <v>2040.423508188082</v>
+      <c r="B12" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="4">
-        <v>0.02801776245389405</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5">
-        <v>7.08751197</v>
+      <c r="B13" s="5">
+        <v>53860.70717579459</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" t="s">
+      <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="5">
-        <v>7.29191612</v>
-      </c>
+      <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="3">
-        <v>7.353382298556016</v>
+      <c r="B16" s="4">
+        <v>-0.02801776245389405</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.02884004300313014</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="2" t="s">
+      <c r="A18" t="s">
         <v>16</v>
+      </c>
+      <c r="B18" s="6">
+        <v>7.08751197</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="6">
+        <v>7.29191612</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="34" customHeight="1">
-      <c r="A21" s="6" t="s">
+      <c r="B21" s="5">
+        <v>2040.423508188082</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
         <v>19</v>
+      </c>
+      <c r="B22" s="5">
+        <v>7.353382298556016</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="34" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -967,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" customWidth="1"/>
@@ -976,158 +1033,163 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0.59985842</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0.66352901</v>
-      </c>
-      <c r="D2" s="4">
-        <v>0.9485436</v>
+      <c r="A2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="3">
-        <v>2019048.41028248</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1699075.79639621</v>
-      </c>
-      <c r="D3" s="3">
-        <v>265066.16180507</v>
+        <v>30</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.59985842</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.66352901</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.9485436</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="3">
-        <v>175113.50965067</v>
-      </c>
-      <c r="C4" s="3">
-        <v>222082.19768122</v>
-      </c>
-      <c r="D4" s="3">
-        <v>672427.37257384</v>
+        <v>31</v>
+      </c>
+      <c r="B4" s="5">
+        <v>2019048.41028248</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1699075.79639621</v>
+      </c>
+      <c r="D4" s="5">
+        <v>265066.16180507</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5">
+        <v>175113.50965067</v>
+      </c>
+      <c r="C5" s="5">
+        <v>222082.19768122</v>
+      </c>
+      <c r="D5" s="5">
+        <v>672427.37257384</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="6">
         <v>17.19944286</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C6" s="6">
         <v>15.00267672</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D6" s="6">
         <v>7.08751197</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-    </row>
     <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="3">
-        <v>1753982.24847741</v>
-      </c>
+      <c r="A8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="3">
+        <v>35</v>
+      </c>
+      <c r="B9" s="5">
+        <v>1753982.24847741</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="5">
         <v>1434009.63459114</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-    </row>
     <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="3">
-        <v>497313.86292317</v>
-      </c>
+      <c r="A12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="3">
+        <v>35</v>
+      </c>
+      <c r="B13" s="5">
+        <v>497313.86292317</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="5">
         <v>450345.17489262</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="48" customHeight="1">
-      <c r="A15" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="2"/>
+    <row r="16" spans="1:4" ht="48" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="3">
-        <v>1227787.573934187</v>
-      </c>
+      <c r="A18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="3"/>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="3">
-        <v>1753982.24847741</v>
+        <v>40</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1227787.573934187</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="3">
+        <v>41</v>
+      </c>
+      <c r="B20" s="5">
+        <v>1753982.24847741</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="5">
         <v>2280176.923020633</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="60" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>37</v>
+    <row r="23" spans="1:2" ht="60" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1137,7 +1199,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7109375" customWidth="1"/>
@@ -1146,97 +1208,102 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0.9485436</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0.9483648</v>
+      <c r="A2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="3">
-        <v>265066.16180507</v>
-      </c>
-      <c r="C3" s="3">
-        <v>264998.26557518</v>
+        <v>30</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.9485436</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.9483648</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="3">
-        <v>672427.37257384</v>
-      </c>
-      <c r="C4" s="3">
-        <v>653587.46218157</v>
+        <v>31</v>
+      </c>
+      <c r="B4" s="5">
+        <v>265066.16180507</v>
+      </c>
+      <c r="C4" s="5">
+        <v>264998.26557518</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5">
-        <v>7.08751197</v>
+        <v>672427.37257384</v>
       </c>
       <c r="C5" s="5">
-        <v>7.29191612</v>
+        <v>653587.46218157</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="3">
+        <v>33</v>
+      </c>
+      <c r="B6" s="6">
+        <v>7.08751197</v>
+      </c>
+      <c r="C6" s="6">
+        <v>7.29191612</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="5">
         <v>4765837.05239493</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C7" s="5">
         <v>4765904.94862482</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="3">
-        <v>18839.91039226996</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="4">
-        <v>0.02801776245389405</v>
+        <v>47</v>
+      </c>
+      <c r="B9" s="5">
+        <v>18839.91039226996</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B10" s="4">
+        <v>0.02801776245389405</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="4">
         <v>0.02884004300313014</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="60" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>44</v>
+    <row r="13" spans="1:3" ht="60" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1246,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1261,683 +1328,688 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" t="s">
+      <c r="E2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
+      <c r="G2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="3">
-        <v>10</v>
-      </c>
-      <c r="E2" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0.36</v>
-      </c>
-      <c r="G2" s="3">
-        <v>15098.26263012</v>
-      </c>
-      <c r="H2" s="3">
-        <v>12092.53736988</v>
-      </c>
-      <c r="I2" s="4">
-        <v>0.4447290028200715</v>
-      </c>
-      <c r="J2" s="4">
-        <v>0.555271</v>
+      <c r="H2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="3">
+        <v>63</v>
+      </c>
+      <c r="D3" s="5">
         <v>10</v>
       </c>
-      <c r="E3" s="3">
-        <v>8.300000000000001</v>
+      <c r="E3" s="5">
+        <v>6.4</v>
       </c>
       <c r="F3" s="4">
-        <v>0.17</v>
-      </c>
-      <c r="G3" s="3">
-        <v>30264.4565287</v>
-      </c>
-      <c r="H3" s="3">
-        <v>11552.1434713</v>
+        <v>0.36</v>
+      </c>
+      <c r="G3" s="5">
+        <v>15098.26263012</v>
+      </c>
+      <c r="H3" s="5">
+        <v>12092.53736988</v>
       </c>
       <c r="I3" s="4">
-        <v>0.2762573588311819</v>
+        <v>0.4447290028200715</v>
       </c>
       <c r="J3" s="4">
-        <v>0.72374264</v>
+        <v>0.555271</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="3">
+        <v>63</v>
+      </c>
+      <c r="D4" s="5">
         <v>10</v>
       </c>
-      <c r="E4" s="3">
-        <v>7</v>
+      <c r="E4" s="5">
+        <v>8.300000000000001</v>
       </c>
       <c r="F4" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G4" s="3">
-        <v>289880.43128787</v>
-      </c>
-      <c r="H4" s="3">
-        <v>9360.56871213</v>
+        <v>0.17</v>
+      </c>
+      <c r="G4" s="5">
+        <v>30264.4565287</v>
+      </c>
+      <c r="H4" s="5">
+        <v>11552.1434713</v>
       </c>
       <c r="I4" s="4">
-        <v>0.03128103673002697</v>
+        <v>0.2762573588311819</v>
       </c>
       <c r="J4" s="4">
-        <v>0.96871896</v>
+        <v>0.72374264</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" t="s">
         <v>63</v>
       </c>
-      <c r="C5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>10</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>7</v>
       </c>
       <c r="F5" s="4">
         <v>0.3</v>
       </c>
-      <c r="G5" s="3">
-        <v>17557.71365225</v>
-      </c>
-      <c r="H5" s="3">
-        <v>5974.28634775</v>
+      <c r="G5" s="5">
+        <v>289880.43128787</v>
+      </c>
+      <c r="H5" s="5">
+        <v>9360.56871213</v>
       </c>
       <c r="I5" s="4">
-        <v>0.2538792430626381</v>
+        <v>0.03128103673002697</v>
       </c>
       <c r="J5" s="4">
-        <v>0.74612076</v>
+        <v>0.96871896</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="3">
+        <v>63</v>
+      </c>
+      <c r="D6" s="5">
         <v>10</v>
       </c>
-      <c r="E6" s="3">
-        <v>8.199999999999999</v>
+      <c r="E6" s="5">
+        <v>7</v>
       </c>
       <c r="F6" s="4">
-        <v>0.18</v>
-      </c>
-      <c r="G6" s="3">
-        <v>13020.00516041</v>
-      </c>
-      <c r="H6" s="3">
-        <v>5957.39483959</v>
+        <v>0.3</v>
+      </c>
+      <c r="G6" s="5">
+        <v>17557.71365225</v>
+      </c>
+      <c r="H6" s="5">
+        <v>5974.28634775</v>
       </c>
       <c r="I6" s="4">
-        <v>0.3139204969906309</v>
+        <v>0.2538792430626381</v>
       </c>
       <c r="J6" s="4">
-        <v>0.6860795</v>
+        <v>0.74612076</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="3">
+        <v>63</v>
+      </c>
+      <c r="D7" s="5">
         <v>10</v>
       </c>
-      <c r="E7" s="3">
-        <v>7</v>
+      <c r="E7" s="5">
+        <v>8.199999999999999</v>
       </c>
       <c r="F7" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G7" s="3">
-        <v>26346.56263092</v>
-      </c>
-      <c r="H7" s="3">
-        <v>5483.43736908</v>
+        <v>0.18</v>
+      </c>
+      <c r="G7" s="5">
+        <v>13020.00516041</v>
+      </c>
+      <c r="H7" s="5">
+        <v>5957.39483959</v>
       </c>
       <c r="I7" s="4">
-        <v>0.1722726160565504</v>
+        <v>0.3139204969906309</v>
       </c>
       <c r="J7" s="4">
-        <v>0.82772738</v>
+        <v>0.6860795</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" t="s">
         <v>67</v>
       </c>
-      <c r="B8" t="s">
-        <v>68</v>
-      </c>
       <c r="C8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="3">
+        <v>63</v>
+      </c>
+      <c r="D8" s="5">
         <v>10</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>7</v>
       </c>
       <c r="F8" s="4">
         <v>0.3</v>
       </c>
-      <c r="G8" s="3">
-        <v>6367.42272522</v>
-      </c>
-      <c r="H8" s="3">
-        <v>5401.57727478</v>
+      <c r="G8" s="5">
+        <v>26346.56263092</v>
+      </c>
+      <c r="H8" s="5">
+        <v>5483.43736908</v>
       </c>
       <c r="I8" s="4">
-        <v>0.458966545567168</v>
+        <v>0.1722726160565504</v>
       </c>
       <c r="J8" s="4">
-        <v>0.54103345</v>
+        <v>0.82772738</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="3">
+        <v>63</v>
+      </c>
+      <c r="D9" s="5">
         <v>10</v>
       </c>
-      <c r="E9" s="3">
-        <v>6.4</v>
+      <c r="E9" s="5">
+        <v>7</v>
       </c>
       <c r="F9" s="4">
-        <v>0.36</v>
-      </c>
-      <c r="G9" s="3">
-        <v>18981.46685885</v>
-      </c>
-      <c r="H9" s="3">
-        <v>5174.53314115</v>
+        <v>0.3</v>
+      </c>
+      <c r="G9" s="5">
+        <v>6367.42272522</v>
+      </c>
+      <c r="H9" s="5">
+        <v>5401.57727478</v>
       </c>
       <c r="I9" s="4">
-        <v>0.2142131619949495</v>
+        <v>0.458966545567168</v>
       </c>
       <c r="J9" s="4">
-        <v>0.78578684</v>
+        <v>0.54103345</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
         <v>63</v>
       </c>
-      <c r="C10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>10</v>
       </c>
-      <c r="E10" s="3">
-        <v>7</v>
+      <c r="E10" s="5">
+        <v>6.4</v>
       </c>
       <c r="F10" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G10" s="3">
-        <v>12481.1744233</v>
-      </c>
-      <c r="H10" s="3">
-        <v>4450.8255767</v>
+        <v>0.36</v>
+      </c>
+      <c r="G10" s="5">
+        <v>18981.46685885</v>
+      </c>
+      <c r="H10" s="5">
+        <v>5174.53314115</v>
       </c>
       <c r="I10" s="4">
-        <v>0.2628647281301678</v>
+        <v>0.2142131619949495</v>
       </c>
       <c r="J10" s="4">
-        <v>0.73713527</v>
+        <v>0.78578684</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="3">
+        <v>63</v>
+      </c>
+      <c r="D11" s="5">
         <v>10</v>
       </c>
-      <c r="E11" s="3">
-        <v>8.300000000000001</v>
+      <c r="E11" s="5">
+        <v>7</v>
       </c>
       <c r="F11" s="4">
-        <v>0.17</v>
-      </c>
-      <c r="G11" s="3">
-        <v>10240.36112165</v>
-      </c>
-      <c r="H11" s="3">
-        <v>4258.93887835</v>
+        <v>0.3</v>
+      </c>
+      <c r="G11" s="5">
+        <v>12481.1744233</v>
+      </c>
+      <c r="H11" s="5">
+        <v>4450.8255767</v>
       </c>
       <c r="I11" s="4">
-        <v>0.2937341029118647</v>
+        <v>0.2628647281301678</v>
       </c>
       <c r="J11" s="4">
-        <v>0.7062659</v>
+        <v>0.73713527</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="3">
+        <v>63</v>
+      </c>
+      <c r="D12" s="5">
         <v>10</v>
       </c>
-      <c r="E12" s="3">
-        <v>7</v>
+      <c r="E12" s="5">
+        <v>8.300000000000001</v>
       </c>
       <c r="F12" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G12" s="3">
-        <v>11396.82583217</v>
-      </c>
-      <c r="H12" s="3">
-        <v>4221.17416783</v>
+        <v>0.17</v>
+      </c>
+      <c r="G12" s="5">
+        <v>10240.36112165</v>
+      </c>
+      <c r="H12" s="5">
+        <v>4258.93887835</v>
       </c>
       <c r="I12" s="4">
-        <v>0.2702762304923806</v>
+        <v>0.2937341029118647</v>
       </c>
       <c r="J12" s="4">
-        <v>0.72972377</v>
+        <v>0.7062659</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="3">
+        <v>63</v>
+      </c>
+      <c r="D13" s="5">
         <v>10</v>
       </c>
-      <c r="E13" s="3">
-        <v>7.4</v>
+      <c r="E13" s="5">
+        <v>7</v>
       </c>
       <c r="F13" s="4">
-        <v>0.26</v>
-      </c>
-      <c r="G13" s="3">
-        <v>55699.04359735</v>
-      </c>
-      <c r="H13" s="3">
-        <v>4137.35640265</v>
+        <v>0.3</v>
+      </c>
+      <c r="G13" s="5">
+        <v>11396.82583217</v>
+      </c>
+      <c r="H13" s="5">
+        <v>4221.17416783</v>
       </c>
       <c r="I13" s="4">
-        <v>0.06914447397654271</v>
+        <v>0.2702762304923806</v>
       </c>
       <c r="J13" s="4">
-        <v>0.93085553</v>
+        <v>0.72972377</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="3">
+        <v>63</v>
+      </c>
+      <c r="D14" s="5">
         <v>10</v>
       </c>
-      <c r="E14" s="3">
-        <v>7</v>
+      <c r="E14" s="5">
+        <v>7.4</v>
       </c>
       <c r="F14" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G14" s="3">
-        <v>35171.36793225</v>
-      </c>
-      <c r="H14" s="3">
-        <v>3708.63206775</v>
+        <v>0.26</v>
+      </c>
+      <c r="G14" s="5">
+        <v>55699.04359735</v>
+      </c>
+      <c r="H14" s="5">
+        <v>4137.35640265</v>
       </c>
       <c r="I14" s="4">
-        <v>0.09538662725694444</v>
+        <v>0.06914447397654271</v>
       </c>
       <c r="J14" s="4">
-        <v>0.90461337</v>
+        <v>0.93085553</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>78</v>
-      </c>
-      <c r="D15" s="3">
+        <v>63</v>
+      </c>
+      <c r="D15" s="5">
         <v>10</v>
       </c>
-      <c r="E15" s="3">
-        <v>8</v>
+      <c r="E15" s="5">
+        <v>7</v>
       </c>
       <c r="F15" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="G15" s="3">
-        <v>60198.80279456</v>
-      </c>
-      <c r="H15" s="3">
-        <v>3634.77320544</v>
+        <v>0.3</v>
+      </c>
+      <c r="G15" s="5">
+        <v>35171.36793225</v>
+      </c>
+      <c r="H15" s="5">
+        <v>3708.63206775</v>
       </c>
       <c r="I15" s="4">
-        <v>0.05694140032888022</v>
+        <v>0.09538662725694444</v>
       </c>
       <c r="J15" s="4">
-        <v>0.9430586</v>
+        <v>0.90461337</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="3">
+        <v>84</v>
+      </c>
+      <c r="D16" s="5">
         <v>10</v>
       </c>
-      <c r="E16" s="3">
-        <v>6.8</v>
+      <c r="E16" s="5">
+        <v>8</v>
       </c>
       <c r="F16" s="4">
-        <v>0.32</v>
-      </c>
-      <c r="G16" s="3">
-        <v>20325.02130884</v>
-      </c>
-      <c r="H16" s="3">
-        <v>3562.97869116</v>
+        <v>0.2</v>
+      </c>
+      <c r="G16" s="5">
+        <v>60198.80279456</v>
+      </c>
+      <c r="H16" s="5">
+        <v>3634.77320544</v>
       </c>
       <c r="I16" s="4">
-        <v>0.1491534951088413</v>
+        <v>0.05694140032888022</v>
       </c>
       <c r="J16" s="4">
-        <v>0.8508465</v>
+        <v>0.9430586</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="3">
+        <v>63</v>
+      </c>
+      <c r="D17" s="5">
         <v>10</v>
       </c>
-      <c r="E17" s="3">
-        <v>7</v>
+      <c r="E17" s="5">
+        <v>6.8</v>
       </c>
       <c r="F17" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="G17" s="3">
-        <v>22390.55209233</v>
-      </c>
-      <c r="H17" s="3">
-        <v>3532.44790767</v>
+        <v>0.32</v>
+      </c>
+      <c r="G17" s="5">
+        <v>20325.02130884</v>
+      </c>
+      <c r="H17" s="5">
+        <v>3562.97869116</v>
       </c>
       <c r="I17" s="4">
-        <v>0.136266940850596</v>
+        <v>0.1491534951088413</v>
       </c>
       <c r="J17" s="4">
-        <v>0.8637330600000001</v>
+        <v>0.8508465</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="3">
+        <v>63</v>
+      </c>
+      <c r="D18" s="5">
         <v>10</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="5">
         <v>7</v>
       </c>
       <c r="F18" s="4">
         <v>0.3</v>
       </c>
-      <c r="G18" s="3">
-        <v>11247.65180345</v>
-      </c>
-      <c r="H18" s="3">
-        <v>3368.34819655</v>
+      <c r="G18" s="5">
+        <v>22390.55209233</v>
+      </c>
+      <c r="H18" s="5">
+        <v>3532.44790767</v>
       </c>
       <c r="I18" s="4">
-        <v>0.2304562258175971</v>
+        <v>0.136266940850596</v>
       </c>
       <c r="J18" s="4">
-        <v>0.76954377</v>
+        <v>0.8637330600000001</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="3">
+        <v>63</v>
+      </c>
+      <c r="D19" s="5">
         <v>10</v>
       </c>
-      <c r="E19" s="3">
-        <v>6.8</v>
+      <c r="E19" s="5">
+        <v>7</v>
       </c>
       <c r="F19" s="4">
-        <v>0.32</v>
-      </c>
-      <c r="G19" s="3">
-        <v>26662.70933894</v>
-      </c>
-      <c r="H19" s="3">
-        <v>3292.49066106</v>
+        <v>0.3</v>
+      </c>
+      <c r="G19" s="5">
+        <v>11247.65180345</v>
+      </c>
+      <c r="H19" s="5">
+        <v>3368.34819655</v>
       </c>
       <c r="I19" s="4">
-        <v>0.1099138266831802</v>
+        <v>0.2304562258175971</v>
       </c>
       <c r="J19" s="4">
-        <v>0.89008617</v>
+        <v>0.76954377</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="3">
+        <v>63</v>
+      </c>
+      <c r="D20" s="5">
         <v>10</v>
       </c>
-      <c r="E20" s="3">
-        <v>8.199999999999999</v>
+      <c r="E20" s="5">
+        <v>6.8</v>
       </c>
       <c r="F20" s="4">
-        <v>0.18</v>
-      </c>
-      <c r="G20" s="3">
-        <v>5603.16526851</v>
-      </c>
-      <c r="H20" s="3">
-        <v>3060.23473149</v>
+        <v>0.32</v>
+      </c>
+      <c r="G20" s="5">
+        <v>26662.70933894</v>
+      </c>
+      <c r="H20" s="5">
+        <v>3292.49066106</v>
       </c>
       <c r="I20" s="4">
-        <v>0.3532371507133458</v>
+        <v>0.1099138266831802</v>
       </c>
       <c r="J20" s="4">
-        <v>0.64676285</v>
+        <v>0.89008617</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="3">
+        <v>63</v>
+      </c>
+      <c r="D21" s="5">
         <v>10</v>
       </c>
-      <c r="E21" s="3">
+      <c r="E21" s="5">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="G21" s="5">
+        <v>5603.16526851</v>
+      </c>
+      <c r="H21" s="5">
+        <v>3060.23473149</v>
+      </c>
+      <c r="I21" s="4">
+        <v>0.3532371507133458</v>
+      </c>
+      <c r="J21" s="4">
+        <v>0.64676285</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" s="5">
+        <v>10</v>
+      </c>
+      <c r="E22" s="5">
         <v>8.6</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F22" s="4">
         <v>0.14</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G22" s="5">
         <v>19776.61545352</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H22" s="5">
         <v>2954.44954648</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I22" s="4">
         <v>0.1299740925680341</v>
       </c>
-      <c r="J21" s="4">
+      <c r="J22" s="4">
         <v>0.87002591</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="48" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>87</v>
+    <row r="24" spans="1:10" ht="48" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A2:J22"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1952,17 +2024,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="48" customHeight="1">
-      <c r="A2" s="6" t="s">
-        <v>89</v>
+      <c r="A2" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="48" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>90</v>
+      <c r="A3" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1981,114 +2053,114 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>93</v>
+      <c r="A1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="34" customHeight="1">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>96</v>
+        <v>101</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="34" customHeight="1">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>96</v>
+        <v>104</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="34" customHeight="1">
       <c r="A4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B4" s="5">
+        <v>105</v>
+      </c>
+      <c r="B4" s="6">
         <v>0.15</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>100</v>
+      <c r="C4" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="34" customHeight="1">
       <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="5">
+        <v>107</v>
+      </c>
+      <c r="B5" s="6">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>102</v>
+      <c r="C5" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="34" customHeight="1">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="34" customHeight="1">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>111</v>
+        <v>116</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="34" customHeight="1">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B9" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
+      <c r="A11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B12" s="4">
         <v>0.3</v>
@@ -2096,7 +2168,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B13" s="4">
         <v>0.32</v>
@@ -2104,7 +2176,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B14" s="4">
         <v>0.3</v>
@@ -2112,7 +2184,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B15" s="4">
         <v>0.17</v>
@@ -2120,7 +2192,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B16" s="4">
         <v>0.22</v>
@@ -2128,7 +2200,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B17" s="4">
         <v>0.17</v>
@@ -2136,7 +2208,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B18" s="4">
         <v>0.26</v>
@@ -2144,7 +2216,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B19" s="4">
         <v>0.18</v>
@@ -2152,7 +2224,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B20" s="4">
         <v>0.18</v>
@@ -2160,7 +2232,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B21" s="4">
         <v>0.3</v>
@@ -2168,7 +2240,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B22" s="4">
         <v>0.14</v>
@@ -2176,7 +2248,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B23" s="4">
         <v>0.36</v>
@@ -2184,7 +2256,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B24" s="4">
         <v>0.14</v>
@@ -2192,7 +2264,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B25" s="4">
         <v>0.2</v>
@@ -2200,7 +2272,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B26" s="4">
         <v>0.14</v>
@@ -2208,13 +2280,13 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B27" s="4">
         <v>0.25</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>132</v>
+      <c r="C27" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2232,47 +2304,47 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="60" customHeight="1">
-      <c r="A2" s="6" t="s">
-        <v>134</v>
+      <c r="A2" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="60" customHeight="1">
-      <c r="A3" s="6" t="s">
-        <v>135</v>
+      <c r="A3" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="60" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>136</v>
+      <c r="A4" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="60" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>137</v>
+      <c r="A5" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="60" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>138</v>
+      <c r="A6" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="60" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>139</v>
+      <c r="A7" s="2" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="60" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>140</v>
+      <c r="A8" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="60" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>141</v>
+      <c r="A9" s="2" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 23: README, aba "Resumo visual" e imagens
- README reescrito: problema, entrega, como funciona (Mermaid), o que foi
  medido (relativos, célula 7/14, fonte ao lado), como sabemos que
  funciona, de onde vêm os dados, limitações verbatim, como rodar
- monthly_report: primeira aba "Resumo visual"
- notebooks/gerar_imagens_readme.py e docs/img/
- documento de negócio: remove "ganho do ML pequeno demais" e afirmações
  de iso-serviço não sustentadas; CLAUDE.md registra a Sprint 24
- docs/teste_do_readme.md: roteiro do teste com um colega
</commit_message>
<xml_diff>
--- a/docs/entregaveis/relatorio_mensal.xlsx
+++ b/docs/entregaveis/relatorio_mensal.xlsx
@@ -7,23 +7,90 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumo executivo" sheetId="1" r:id="rId1"/>
-    <sheet name="Andar 1 - Correção de cadastro" sheetId="2" r:id="rId2"/>
-    <sheet name="Andar 2 - Refinamento do modelo" sheetId="3" r:id="rId3"/>
-    <sheet name="Itens sangrando margem" sheetId="4" r:id="rId4"/>
-    <sheet name="Taxa de aceitação" sheetId="5" r:id="rId5"/>
-    <sheet name="Premissas" sheetId="6" r:id="rId6"/>
-    <sheet name="Limitações" sheetId="7" r:id="rId7"/>
+    <sheet name="Resumo visual" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumo executivo" sheetId="2" r:id="rId2"/>
+    <sheet name="Andar 1 - Correção de cadastro" sheetId="3" r:id="rId3"/>
+    <sheet name="Andar 2 - Refinamento do modelo" sheetId="4" r:id="rId4"/>
+    <sheet name="Itens sangrando margem" sheetId="5" r:id="rId5"/>
+    <sheet name="Taxa de aceitação" sheetId="6" r:id="rId6"/>
+    <sheet name="Premissas" sheetId="7" r:id="rId7"/>
+    <sheet name="Limitações" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Itens sangrando margem'!$A$2:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Itens sangrando margem'!$A$2:$J$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="169">
+  <si>
+    <t>RELATÓRIO MENSAL -- RESUMO</t>
+  </si>
+  <si>
+    <t>Backtest de 277 dias sobre o dado do Favorita, célula lead time 7 / revisão 14. Só números relativos; R$ nas outras abas é ilustrativo (preço uniforme de R$ 10, margem arbitrada).</t>
+  </si>
+  <si>
+    <t>NÍVEL DE SERVIÇO</t>
+  </si>
+  <si>
+    <t>60% → 95%</t>
+  </si>
+  <si>
+    <t>De cada 100 unidades que o cliente quis comprar, 60 eram atendidas com o cadastro desatualizado e 95 depois de recalibrar (Andar 1).</t>
+  </si>
+  <si>
+    <t>Andar 2: motor 94,8% contra 94,9% do baseline recalibrado -- mesmo serviço, por construção (iso-serviço).</t>
+  </si>
+  <si>
+    <t>Fonte: results/baseline_desatualizado (calibrado_lt3_rp7), results/sensibilidade_dirigida/lt7_rp14 e results/iso_servico (alpha 0,66).</t>
+  </si>
+  <si>
+    <t>CAPITAL PARADO</t>
+  </si>
+  <si>
+    <t>Capital médio empregado para sair de 60% para 95% de serviço (Andar 1): servir mais exige estocar mais, não menos.</t>
+  </si>
+  <si>
+    <t>Andar 2: −2,8% no mesmo serviço (motor contra o baseline recalibrado).</t>
+  </si>
+  <si>
+    <t>Fonte: capital_medio_rs de results/baseline_desatualizado, results/sensibilidade_dirigida/lt7_rp14 e results/iso_servico.</t>
+  </si>
+  <si>
+    <t>MARGEM POR REAL INVESTIDO</t>
+  </si>
+  <si>
+    <t>Andar 2: motor contra o baseline já recalibrado, no mesmo nível de serviço. É o ganho do modelo; o Andar 1 (recalibrar o cadastro) é a parte maior da conta.</t>
+  </si>
+  <si>
+    <t>Fonte: decision_metric de results/iso_servico e results/sensibilidade_dirigida/lt7_rp14.</t>
+  </si>
+  <si>
+    <t>Dados dos gráficos</t>
+  </si>
+  <si>
+    <t>cenário</t>
+  </si>
+  <si>
+    <t>nível de serviço</t>
+  </si>
+  <si>
+    <t>capital (índice)</t>
+  </si>
+  <si>
+    <t>ERP desatualizado</t>
+  </si>
+  <si>
+    <t>ERP recalibrado</t>
+  </si>
+  <si>
+    <t>Motor (braço 2)</t>
+  </si>
+  <si>
+    <t>Capital: índice 100 = baseline recalibrado. Perda evitada e taxa de aceitação não são medidas -- ver aba Limitações.</t>
+  </si>
   <si>
     <t>RELATÓRIO MENSAL EM R$ -- MOTOR DE DECISÃO DE COMPRA</t>
   </si>
@@ -113,9 +180,6 @@
   </si>
   <si>
     <t>recalibrado</t>
-  </si>
-  <si>
-    <t>nível de serviço</t>
   </si>
   <si>
     <t>ruptura_rs (total do período)</t>
@@ -473,15 +537,56 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="+0%;-0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF6B6B6B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="32"/>
+      <color rgb="FF0B0B0B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF6B6B6B"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -544,16 +649,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,6 +683,349 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" baseline="0"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1000" baseline="0"/>
+              <a:t>Nível de serviço (%)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Nível de serviço (%)</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="0"/>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Resumo visual'!$A$44:$A$46</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>ERP desatualizado</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>ERP recalibrado</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Motor (braço 2)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Resumo visual'!$B$44:$B$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.59985842</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.9485436</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.9483648</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1.0"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" baseline="0"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1000" baseline="0"/>
+              <a:t>Capital médio empregado (índice, 100 = baseline recalibrado)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Capital médio empregado (índice, 100 = baseline recalibrado)</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:numFmt formatCode="0" sourceLinked="0"/>
+            <c:showVal val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Resumo visual'!$A$44:$A$46</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>ERP desatualizado</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>ERP recalibrado</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Motor (braço 2)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Resumo visual'!$C$44:$C$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>26.04199602707883</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>97.19822375461059</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50020001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50020002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="120"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -848,6 +1313,155 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C47"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="46.7109375" customWidth="1"/>
+    <col min="2" max="3" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="44" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="46" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="32" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="32" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="30" customHeight="1">
+      <c r="A8" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="46" customHeight="1">
+      <c r="A11" s="6">
+        <v>2.839951434445293</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="32" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="32" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="30" customHeight="1">
+      <c r="A14" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="46" customHeight="1">
+      <c r="A17" s="7">
+        <v>0.02884004300313014</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="32" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="30" customHeight="1">
+      <c r="A19" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>18</v>
+      </c>
+      <c r="B44" s="10">
+        <v>0.59985842</v>
+      </c>
+      <c r="C44" s="11">
+        <v>26.04199602707883</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" s="10">
+        <v>0.9485436</v>
+      </c>
+      <c r="C45" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="10">
+        <v>0.9483648</v>
+      </c>
+      <c r="C46" s="11">
+        <v>97.19822375461059</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="30" customHeight="1">
+      <c r="A47" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -856,165 +1470,165 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="8" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="30" customHeight="1">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
+      <c r="A3" s="12" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3"/>
+      <c r="A5" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="9"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4">
+        <v>26</v>
+      </c>
+      <c r="B6" s="10">
         <v>0.59985842</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4">
+        <v>27</v>
+      </c>
+      <c r="B7" s="10">
         <v>0.9485436</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4">
+        <v>28</v>
+      </c>
+      <c r="B8" s="10">
         <v>0.8687172826292039</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4">
+        <v>29</v>
+      </c>
+      <c r="B9" s="10">
         <v>2.839951434445293</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>8</v>
+      <c r="A10" s="12" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5">
+        <v>31</v>
+      </c>
+      <c r="B11" s="13">
         <v>189961.9763693946</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="5">
+        <v>34</v>
+      </c>
+      <c r="B13" s="13">
         <v>53860.70717579459</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="3"/>
+      <c r="A15" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="9"/>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="4">
+        <v>36</v>
+      </c>
+      <c r="B16" s="10">
         <v>-0.02801776245389405</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="4">
+        <v>37</v>
+      </c>
+      <c r="B17" s="10">
         <v>0.02884004300313014</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="6">
+        <v>38</v>
+      </c>
+      <c r="B18" s="11">
         <v>7.08751197</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6">
+        <v>39</v>
+      </c>
+      <c r="B19" s="11">
         <v>7.29191612</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>8</v>
+      <c r="A20" s="12" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="5">
+        <v>40</v>
+      </c>
+      <c r="B21" s="13">
         <v>2040.423508188082</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="5">
+        <v>41</v>
+      </c>
+      <c r="B22" s="13">
         <v>7.353382298556016</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>21</v>
+      <c r="A24" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="34" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>24</v>
+      <c r="A27" s="12" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1022,7 +1636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1032,164 +1646,164 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
+      <c r="A1" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>29</v>
+      <c r="A2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="4">
+        <v>16</v>
+      </c>
+      <c r="B3" s="10">
         <v>0.59985842</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="10">
         <v>0.66352901</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="10">
         <v>0.9485436</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="5">
+        <v>52</v>
+      </c>
+      <c r="B4" s="13">
         <v>2019048.41028248</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="13">
         <v>1699075.79639621</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="13">
         <v>265066.16180507</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="5">
+        <v>53</v>
+      </c>
+      <c r="B5" s="13">
         <v>175113.50965067</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="13">
         <v>222082.19768122</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="13">
         <v>672427.37257384</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="6">
+        <v>54</v>
+      </c>
+      <c r="B6" s="11">
         <v>17.19944286</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="11">
         <v>15.00267672</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="11">
         <v>7.08751197</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="A8" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="5">
+        <v>56</v>
+      </c>
+      <c r="B9" s="13">
         <v>1753982.24847741</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="5">
+        <v>57</v>
+      </c>
+      <c r="B10" s="13">
         <v>1434009.63459114</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="A12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="5">
+        <v>56</v>
+      </c>
+      <c r="B13" s="13">
         <v>497313.86292317</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="5">
+        <v>57</v>
+      </c>
+      <c r="B14" s="13">
         <v>450345.17489262</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="48" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>38</v>
+      <c r="A16" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="3"/>
+      <c r="A18" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="9"/>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="5">
+        <v>61</v>
+      </c>
+      <c r="B19" s="13">
         <v>1227787.573934187</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="5">
+        <v>62</v>
+      </c>
+      <c r="B20" s="13">
         <v>1753982.24847741</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="5">
+        <v>63</v>
+      </c>
+      <c r="B21" s="13">
         <v>2280176.923020633</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="60" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>43</v>
+      <c r="A23" s="12" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1197,7 +1811,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1207,103 +1821,103 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
+      <c r="A1" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>45</v>
+      <c r="A2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="4">
+        <v>16</v>
+      </c>
+      <c r="B3" s="10">
         <v>0.9485436</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="10">
         <v>0.9483648</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="5">
+        <v>52</v>
+      </c>
+      <c r="B4" s="13">
         <v>265066.16180507</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="13">
         <v>264998.26557518</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="5">
+        <v>53</v>
+      </c>
+      <c r="B5" s="13">
         <v>672427.37257384</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="13">
         <v>653587.46218157</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="6">
+        <v>54</v>
+      </c>
+      <c r="B6" s="11">
         <v>7.08751197</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="11">
         <v>7.29191612</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="5">
+        <v>67</v>
+      </c>
+      <c r="B7" s="13">
         <v>4765837.05239493</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="13">
         <v>4765904.94862482</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="5">
+        <v>68</v>
+      </c>
+      <c r="B9" s="13">
         <v>18839.91039226996</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" s="4">
+        <v>69</v>
+      </c>
+      <c r="B10" s="10">
         <v>0.02801776245389405</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="4">
+        <v>70</v>
+      </c>
+      <c r="B11" s="10">
         <v>0.02884004300313014</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="60" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>50</v>
+      <c r="A13" s="12" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1311,7 +1925,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1327,685 +1941,685 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
+      <c r="A1" s="12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>60</v>
+      <c r="A2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="5">
+        <v>84</v>
+      </c>
+      <c r="D3" s="13">
         <v>10</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="13">
         <v>6.4</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="10">
         <v>0.36</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="13">
         <v>15098.26263012</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="13">
         <v>12092.53736988</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="10">
         <v>0.4447290028200715</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="10">
         <v>0.555271</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="5">
+        <v>84</v>
+      </c>
+      <c r="D4" s="13">
         <v>10</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="13">
         <v>8.300000000000001</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="10">
         <v>0.17</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="13">
         <v>30264.4565287</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="13">
         <v>11552.1434713</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="10">
         <v>0.2762573588311819</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="10">
         <v>0.72374264</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="5">
+        <v>84</v>
+      </c>
+      <c r="D5" s="13">
         <v>10</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="13">
         <v>7</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="10">
         <v>0.3</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="13">
         <v>289880.43128787</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="13">
         <v>9360.56871213</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="10">
         <v>0.03128103673002697</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="10">
         <v>0.96871896</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="5">
+        <v>84</v>
+      </c>
+      <c r="D6" s="13">
         <v>10</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="13">
         <v>7</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="10">
         <v>0.3</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="13">
         <v>17557.71365225</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="13">
         <v>5974.28634775</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="10">
         <v>0.2538792430626381</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="10">
         <v>0.74612076</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="5">
+        <v>84</v>
+      </c>
+      <c r="D7" s="13">
         <v>10</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="13">
         <v>8.199999999999999</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="10">
         <v>0.18</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="13">
         <v>13020.00516041</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="13">
         <v>5957.39483959</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="10">
         <v>0.3139204969906309</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="10">
         <v>0.6860795</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="5">
+        <v>84</v>
+      </c>
+      <c r="D8" s="13">
         <v>10</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="13">
         <v>7</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="10">
         <v>0.3</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="13">
         <v>26346.56263092</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="13">
         <v>5483.43736908</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="10">
         <v>0.1722726160565504</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="10">
         <v>0.82772738</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="5">
+        <v>84</v>
+      </c>
+      <c r="D9" s="13">
         <v>10</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="13">
         <v>7</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="10">
         <v>0.3</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="13">
         <v>6367.42272522</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="13">
         <v>5401.57727478</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="10">
         <v>0.458966545567168</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="10">
         <v>0.54103345</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="5">
+        <v>84</v>
+      </c>
+      <c r="D10" s="13">
         <v>10</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="13">
         <v>6.4</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="10">
         <v>0.36</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="13">
         <v>18981.46685885</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="13">
         <v>5174.53314115</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="10">
         <v>0.2142131619949495</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="10">
         <v>0.78578684</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" s="5">
+        <v>84</v>
+      </c>
+      <c r="D11" s="13">
         <v>10</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="13">
         <v>7</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="10">
         <v>0.3</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="13">
         <v>12481.1744233</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="13">
         <v>4450.8255767</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="10">
         <v>0.2628647281301678</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="10">
         <v>0.73713527</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="5">
+        <v>84</v>
+      </c>
+      <c r="D12" s="13">
         <v>10</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="13">
         <v>8.300000000000001</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="10">
         <v>0.17</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="13">
         <v>10240.36112165</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="13">
         <v>4258.93887835</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="10">
         <v>0.2937341029118647</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="10">
         <v>0.7062659</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
-      </c>
-      <c r="D13" s="5">
+        <v>84</v>
+      </c>
+      <c r="D13" s="13">
         <v>10</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="13">
         <v>7</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="10">
         <v>0.3</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="13">
         <v>11396.82583217</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="13">
         <v>4221.17416783</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="10">
         <v>0.2702762304923806</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="10">
         <v>0.72972377</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="5">
+        <v>84</v>
+      </c>
+      <c r="D14" s="13">
         <v>10</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="13">
         <v>7.4</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="10">
         <v>0.26</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="13">
         <v>55699.04359735</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="13">
         <v>4137.35640265</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="10">
         <v>0.06914447397654271</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="10">
         <v>0.93085553</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
-      </c>
-      <c r="D15" s="5">
+        <v>84</v>
+      </c>
+      <c r="D15" s="13">
         <v>10</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="13">
         <v>7</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="10">
         <v>0.3</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="13">
         <v>35171.36793225</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="13">
         <v>3708.63206775</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="10">
         <v>0.09538662725694444</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="10">
         <v>0.90461337</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="5">
+        <v>105</v>
+      </c>
+      <c r="D16" s="13">
         <v>10</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="13">
         <v>8</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="10">
         <v>0.2</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="13">
         <v>60198.80279456</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="13">
         <v>3634.77320544</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="10">
         <v>0.05694140032888022</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="10">
         <v>0.9430586</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="5">
+        <v>84</v>
+      </c>
+      <c r="D17" s="13">
         <v>10</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="13">
         <v>6.8</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="10">
         <v>0.32</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="13">
         <v>20325.02130884</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="13">
         <v>3562.97869116</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="10">
         <v>0.1491534951088413</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="10">
         <v>0.8508465</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="5">
+        <v>84</v>
+      </c>
+      <c r="D18" s="13">
         <v>10</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="13">
         <v>7</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="10">
         <v>0.3</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="13">
         <v>22390.55209233</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="13">
         <v>3532.44790767</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="10">
         <v>0.136266940850596</v>
       </c>
-      <c r="J18" s="4">
+      <c r="J18" s="10">
         <v>0.8637330600000001</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="5">
+        <v>84</v>
+      </c>
+      <c r="D19" s="13">
         <v>10</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="13">
         <v>7</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="10">
         <v>0.3</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="13">
         <v>11247.65180345</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="13">
         <v>3368.34819655</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="10">
         <v>0.2304562258175971</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19" s="10">
         <v>0.76954377</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="5">
+        <v>84</v>
+      </c>
+      <c r="D20" s="13">
         <v>10</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="13">
         <v>6.8</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="10">
         <v>0.32</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="13">
         <v>26662.70933894</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="13">
         <v>3292.49066106</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I20" s="10">
         <v>0.1099138266831802</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J20" s="10">
         <v>0.89008617</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
-      </c>
-      <c r="D21" s="5">
+        <v>84</v>
+      </c>
+      <c r="D21" s="13">
         <v>10</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="13">
         <v>8.199999999999999</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="10">
         <v>0.18</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="13">
         <v>5603.16526851</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="13">
         <v>3060.23473149</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I21" s="10">
         <v>0.3532371507133458</v>
       </c>
-      <c r="J21" s="4">
+      <c r="J21" s="10">
         <v>0.64676285</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
-      </c>
-      <c r="D22" s="5">
+        <v>105</v>
+      </c>
+      <c r="D22" s="13">
         <v>10</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="13">
         <v>8.6</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="10">
         <v>0.14</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="13">
         <v>19776.61545352</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="13">
         <v>2954.44954648</v>
       </c>
-      <c r="I22" s="4">
+      <c r="I22" s="10">
         <v>0.1299740925680341</v>
       </c>
-      <c r="J22" s="4">
+      <c r="J22" s="10">
         <v>0.87002591</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="48" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>93</v>
+      <c r="A24" s="12" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2014,7 +2628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2023,18 +2637,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>94</v>
+      <c r="A1" s="8" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="48" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>95</v>
+      <c r="A2" s="12" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="48" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>96</v>
+      <c r="A3" s="12" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2042,7 +2656,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2053,240 +2667,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>99</v>
+      <c r="A1" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="34" customHeight="1">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>102</v>
+        <v>122</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="34" customHeight="1">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>102</v>
+        <v>125</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="34" customHeight="1">
       <c r="A4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="6">
+        <v>126</v>
+      </c>
+      <c r="B4" s="11">
         <v>0.15</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>106</v>
+      <c r="C4" s="12" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="34" customHeight="1">
       <c r="A5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5" s="6">
+        <v>128</v>
+      </c>
+      <c r="B5" s="11">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>108</v>
+      <c r="C5" s="12" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="34" customHeight="1">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>111</v>
+        <v>131</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="34" customHeight="1">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>114</v>
+        <v>134</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" customHeight="1">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>117</v>
+        <v>137</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="34" customHeight="1">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>120</v>
+        <v>140</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="A11" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>122</v>
-      </c>
-      <c r="B12" s="4">
+        <v>143</v>
+      </c>
+      <c r="B12" s="10">
         <v>0.3</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>123</v>
-      </c>
-      <c r="B13" s="4">
+        <v>144</v>
+      </c>
+      <c r="B13" s="10">
         <v>0.32</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>124</v>
-      </c>
-      <c r="B14" s="4">
+        <v>145</v>
+      </c>
+      <c r="B14" s="10">
         <v>0.3</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>125</v>
-      </c>
-      <c r="B15" s="4">
+        <v>146</v>
+      </c>
+      <c r="B15" s="10">
         <v>0.17</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>126</v>
-      </c>
-      <c r="B16" s="4">
+        <v>147</v>
+      </c>
+      <c r="B16" s="10">
         <v>0.22</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>127</v>
-      </c>
-      <c r="B17" s="4">
+        <v>148</v>
+      </c>
+      <c r="B17" s="10">
         <v>0.17</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>128</v>
-      </c>
-      <c r="B18" s="4">
+        <v>149</v>
+      </c>
+      <c r="B18" s="10">
         <v>0.26</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>129</v>
-      </c>
-      <c r="B19" s="4">
+        <v>150</v>
+      </c>
+      <c r="B19" s="10">
         <v>0.18</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>130</v>
-      </c>
-      <c r="B20" s="4">
+        <v>151</v>
+      </c>
+      <c r="B20" s="10">
         <v>0.18</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="4">
+        <v>152</v>
+      </c>
+      <c r="B21" s="10">
         <v>0.3</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>132</v>
-      </c>
-      <c r="B22" s="4">
+        <v>153</v>
+      </c>
+      <c r="B22" s="10">
         <v>0.14</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>133</v>
-      </c>
-      <c r="B23" s="4">
+        <v>154</v>
+      </c>
+      <c r="B23" s="10">
         <v>0.36</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>134</v>
-      </c>
-      <c r="B24" s="4">
+        <v>155</v>
+      </c>
+      <c r="B24" s="10">
         <v>0.14</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>135</v>
-      </c>
-      <c r="B25" s="4">
+        <v>156</v>
+      </c>
+      <c r="B25" s="10">
         <v>0.2</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>136</v>
-      </c>
-      <c r="B26" s="4">
+        <v>157</v>
+      </c>
+      <c r="B26" s="10">
         <v>0.14</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>137</v>
-      </c>
-      <c r="B27" s="4">
+        <v>158</v>
+      </c>
+      <c r="B27" s="10">
         <v>0.25</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>138</v>
+      <c r="C27" s="12" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -2294,7 +2908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2303,48 +2917,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>139</v>
+      <c r="A1" s="8" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="60" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>140</v>
+      <c r="A2" s="12" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="60" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>141</v>
+      <c r="A3" s="12" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="60" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>142</v>
+      <c r="A4" s="12" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="60" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>143</v>
+      <c r="A5" s="12" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="60" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>144</v>
+      <c r="A6" s="12" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="60" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>145</v>
+      <c r="A7" s="12" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="60" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>146</v>
+      <c r="A8" s="12" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="60" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>147</v>
+      <c r="A9" s="12" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>